<commit_message>
Update spec document to match the current PII-check app
The spec still described the original chat app (conversation history,
model-switching UI, POST /api/chat) even though that feature was
removed and replaced with file-upload PII checking several iterations
ago. Rewrite every sheet to match what's actually implemented: the
7 supported file formats, the 4 detection methods, the fixed single
model, the audit logging feature, Google Workspace SSO, and Docker/
Kubernetes deployment. Keeps the original workbook's structure,
fonts, and styling; adds a 2.0 revision history entry summarizing the
change instead of overwriting the 1.0 entry.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NcsoDYnHXuDZWQAHCjJCPn
</commit_message>
<xml_diff>
--- a/docs/Local_Gemma_Chat_仕様書.xlsx
+++ b/docs/Local_Gemma_Chat_仕様書.xlsx
@@ -83,7 +83,7 @@
       <sz val="14"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -100,6 +100,16 @@
       <patternFill patternType="solid">
         <fgColor rgb="00F2F2F2"/>
         <bgColor rgb="00F2F2F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F2F2F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9E1F2"/>
       </patternFill>
     </fill>
   </fills>
@@ -129,7 +139,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -166,6 +176,21 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -532,7 +557,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A3:H21"/>
+  <dimension ref="A3:H22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -543,7 +568,7 @@
     <row r="3">
       <c r="B3" s="1" t="inlineStr">
         <is>
-          <t>ローカルLLMチャットアプリケーション</t>
+          <t>個人情報チェックアプリケーション</t>
         </is>
       </c>
     </row>
@@ -557,7 +582,7 @@
     <row r="6" ht="30" customHeight="1">
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>Ollama上で動作するGemmaモデルとチャットできる、ローカル環境向けWebアプリケーションの仕様書</t>
+          <t>Ollama上で動作するGemmaモデルと正規表現によるパターンマッチングを組み合わせ、アップロードされたファイルにマスキング漏れの個人情報が残っていないかを検出する、社内向けWebアプリケーションの仕様書</t>
         </is>
       </c>
     </row>
@@ -581,7 +606,7 @@
       </c>
       <c r="C10" s="6" t="inlineStr">
         <is>
-          <t>ローカルLLMチャットアプリケーション 仕様書</t>
+          <t>個人情報チェックアプリケーション 仕様書</t>
         </is>
       </c>
     </row>
@@ -605,7 +630,7 @@
       </c>
       <c r="C12" s="6" t="inlineStr">
         <is>
-          <t>1.0</t>
+          <t>2.0</t>
         </is>
       </c>
     </row>
@@ -617,7 +642,7 @@
       </c>
       <c r="C13" s="6" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
@@ -707,6 +732,23 @@
       <c r="C21" s="10" t="inlineStr">
         <is>
           <t>初版作成(チャット機能・会話履歴保存・モデル切替UI・Docker対応を反映)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="13" t="inlineStr">
+        <is>
+          <t>2.0</t>
+        </is>
+      </c>
+      <c r="B22" s="13" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="C22" s="13" t="inlineStr">
+        <is>
+          <t>チャット機能を廃止し、個人情報チェック専用アプリに全面刷新。対応ファイル形式を.xlsx/.pdfから.docx/.pptx/.csv/.txt/.jsonへ拡張し、正規表現(敬称なし人名検出等)・列見出し/キー名検出・ラベル付きテキスト検出・AI(Gemma)検出の4方式による15種類の個人情報検出を実装。UIを全面リデザインし、利用モデルを単一固定化(既定gemma4:e4b)。アップロード監査ログ(日次ローテーション・既定90日保持)、Google Workspace SSO(oauth2-proxy)連携、Kubernetesデプロイ対応を追加。</t>
         </is>
       </c>
     </row>
@@ -741,80 +783,83 @@
       </c>
     </row>
     <row r="3" ht="20" customHeight="1">
-      <c r="A3" s="12" t="inlineStr">
+      <c r="A3" s="15" t="inlineStr">
         <is>
           <t>目的</t>
         </is>
       </c>
       <c r="B3" s="13" t="inlineStr">
         <is>
-          <t>インターネットや外部SaaSに接続することなく、ローカル環境で稼働するLLM(Gemma)とチャットできるWebアプリケーションを提供する。</t>
+          <t>社内で取り扱うファイル(xlsx/pdf/docx/pptx/csv/txt/json)に、マスキング漏れの個人情報が残っていないかを、外部サービスに一切データを送信することなくローカル環境で確認できるWebアプリケーションを提供する。</t>
         </is>
       </c>
     </row>
     <row r="4" ht="20" customHeight="1">
-      <c r="A4" s="12" t="inlineStr">
+      <c r="A4" s="15" t="inlineStr">
         <is>
           <t>背景</t>
         </is>
       </c>
       <c r="B4" s="13" t="inlineStr">
         <is>
-          <t>クラウドLLM APIには通信コスト・データ送信によるプライバシー懸念・利用料金が伴う。Ollamaを用いてモデルをローカル実行することで、これらを回避しつつ手軽にLLMを試用・利用できる環境を整備する。</t>
+          <t>マスキング作業の確認を目視のみに頼ると見落としが発生しやすい。一方でクラウドAPIに文書を送信してチェックする方法は、個人情報を含む文書自体を外部に送信することになりプライバシー上のリスクが大きい。Ollamaでローカル実行するLLM(Gemma)と正規表現によるパターンマッチングを組み合わせることで、データを外部に出さずにダブルチェックできる環境を整備する。</t>
         </is>
       </c>
     </row>
     <row r="5" ht="20" customHeight="1">
-      <c r="A5" s="12" t="inlineStr">
+      <c r="A5" s="15" t="inlineStr">
         <is>
           <t>想定利用者</t>
         </is>
       </c>
       <c r="B5" s="13" t="inlineStr">
         <is>
-          <t>個人の検証利用、および社内での技術検証・PoC用途。</t>
+          <t>社内で個人情報を含む可能性のある文書を取り扱う担当者。社内ネットワーク/VPN限定・Google Workspace SSO連携により、複数の社員が共有して利用することを想定。</t>
         </is>
       </c>
     </row>
     <row r="6" ht="60" customHeight="1">
-      <c r="A6" s="12" t="inlineStr">
+      <c r="A6" s="15" t="inlineStr">
         <is>
           <t>スコープ(対象)</t>
         </is>
       </c>
       <c r="B6" s="13" t="inlineStr">
         <is>
-          <t>・チャットUI(ストリーミング表示)
-・会話履歴の保存と複数会話の管理
-・複数モデルの切り替えUI
-・Dockerによる環境構築の簡易化</t>
+          <t>・.xlsx/.pdf/.docx/.pptx/.csv/.txt/.jsonファイルのアップロードによる個人情報チェック
+・正規表現パターン検出・列見出し/キー名検出・ラベル付きテキスト検出・AI(Gemma)検出の4方式による15種類の個人情報の検出
+・検出結果のカテゴリ別表示
+・アップロード監査ログの記録(日次ローテーション・保持期間管理)
+・Google Workspace SSO連携による社内向けアクセス制御(本番構成、任意)
+・Docker Compose / Kubernetesによる環境構築</t>
         </is>
       </c>
     </row>
     <row r="7" ht="60" customHeight="1">
-      <c r="A7" s="12" t="inlineStr">
+      <c r="A7" s="15" t="inlineStr">
         <is>
           <t>スコープ外(対象外)</t>
         </is>
       </c>
       <c r="B7" s="13" t="inlineStr">
         <is>
-          <t>・ユーザー認証/アクセス制御
-・複数ユーザーでの会話履歴の共有
-・サーバーサイド(DB等)への会話履歴の永続化
+          <t>・チャット等の対話的な利用機能(初期バージョンに存在したが削除済み)
+・画像のみのPDF、画像内の文字に対するOCR
+・検出された個人情報の自動マスキング/修正(検出のみ行い、修正は行わない)
+・アプリ自体でのユーザー認証機能の実装(認証はoauth2-proxy等の外部コンポーネントに委譲)
 ・モデルのファインチューニング機能</t>
         </is>
       </c>
     </row>
     <row r="8" ht="20" customHeight="1">
-      <c r="A8" s="12" t="inlineStr">
+      <c r="A8" s="15" t="inlineStr">
         <is>
           <t>使用LLM</t>
         </is>
       </c>
       <c r="B8" s="13" t="inlineStr">
         <is>
-          <t>Gemma(Ollama経由)。既定モデル名は "gemma4" だが、Ollamaのモデルライブラリに存在しない場合は "gemma3" 等の実在するタグに読み替える(詳細はシート「7. 今後の課題」参照)。</t>
+          <t>Gemma 4(Ollama経由)。既定モデル名は"gemma4:e4b"(軽量なオンデバイス向けタグ)。アプリ全体で1つのモデルに固定され、環境変数MODEL_NAMEで変更できる(画面上での切り替えはできない)。</t>
         </is>
       </c>
     </row>
@@ -829,7 +874,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -847,157 +892,265 @@
       </c>
     </row>
     <row r="3" ht="22" customHeight="1">
-      <c r="A3" s="8" t="inlineStr">
+      <c r="A3" s="16" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="B3" s="8" t="inlineStr">
+      <c r="B3" s="16" t="inlineStr">
         <is>
           <t>機能名</t>
         </is>
       </c>
-      <c r="C3" s="8" t="inlineStr">
+      <c r="C3" s="16" t="inlineStr">
         <is>
           <t>概要</t>
         </is>
       </c>
-      <c r="D3" s="8" t="inlineStr">
+      <c r="D3" s="16" t="inlineStr">
         <is>
           <t>詳細仕様</t>
         </is>
       </c>
-      <c r="E3" s="8" t="inlineStr">
+      <c r="E3" s="16" t="inlineStr">
         <is>
           <t>実装状況</t>
         </is>
       </c>
     </row>
     <row r="4" ht="56" customHeight="1">
-      <c r="A4" s="9" t="n">
+      <c r="A4" s="17" t="n">
         <v>1</v>
       </c>
-      <c r="B4" s="9" t="inlineStr">
-        <is>
-          <t>チャット(ストリーミング応答)</t>
+      <c r="B4" s="17" t="inlineStr">
+        <is>
+          <t>ファイルアップロード&amp;個人情報チェック</t>
         </is>
       </c>
       <c r="C4" s="10" t="inlineStr">
         <is>
-          <t>ユーザーが入力したメッセージに対し、Gemmaモデルの応答をリアルタイムに表示する。</t>
+          <t>マスキング済みファイルをアップロードし、個人情報が残っていないかチェックする。</t>
         </is>
       </c>
       <c r="D4" s="10" t="inlineStr">
         <is>
-          <t>ブラウザは会話履歴(role/content配列)をサーバーの POST /api/chat に送信する。サーバーは Ollama の POST /api/chat (stream: true) に転送し、返却されるNDJSONストリームを1行ずつパースして生成テキスト部分のみをチャンク転送(chunked)でブラウザへ流す。ブラウザは受信したチャンクを逐次画面に反映する。Enterキーで送信、Shift+Enterで改行。</t>
-        </is>
-      </c>
-      <c r="E4" s="9" t="inlineStr">
+          <t>ブラウザはドラッグ&amp;ドロップまたはファイル選択で.xlsx/.pdf/.docx/.pptx/.csv/.txt/.json(最大50MB)のいずれかを選択し、POST /api/pii-check (multipart/form-data) に送信する。サーバーは拡張子に応じてexceljs/pdf-parse/mammoth/jszip/csv-parse等で本文を抽出し、15種類の個人情報(人物名・フリガナ・住所地名・企業名組織名・日付・時刻・金額・数量・電話番号・メールアドレス・マイナンバー・郵便番号・クレジットカード番号・銀行口座番号・パスポート番号)の有無を判定する。テキストを一切抽出できなかった場合(空ファイル・画像のみのPDF等)は「判定できませんでした」として区別して表示する。</t>
+        </is>
+      </c>
+      <c r="E4" s="17" t="inlineStr">
         <is>
           <t>実装済み</t>
         </is>
       </c>
     </row>
     <row r="5" ht="42" customHeight="1">
-      <c r="A5" s="9" t="n">
+      <c r="A5" s="17" t="n">
         <v>2</v>
       </c>
-      <c r="B5" s="9" t="inlineStr">
-        <is>
-          <t>会話履歴の保存</t>
+      <c r="B5" s="17" t="inlineStr">
+        <is>
+          <t>正規表現によるパターン検出</t>
         </is>
       </c>
       <c r="C5" s="10" t="inlineStr">
         <is>
-          <t>複数の会話(チャット)をブラウザ内に保存し、後から呼び出せるようにする。</t>
+          <t>代表的な書式の個人情報を正規表現でサーバー側検出する。</t>
         </is>
       </c>
       <c r="D5" s="10" t="inlineStr">
         <is>
-          <t>ブラウザの localStorage に会話一覧をJSON配列として保存する(キー: gemma-chat-conversations)。各会話は id・title・model・messages・updatedAt を持つ。画面左のサイドバーから新規作成・選択・削除が可能。タイトルは最初のユーザー発言(先頭30文字)から自動生成する。</t>
-        </is>
-      </c>
-      <c r="E5" s="9" t="inlineStr">
+          <t>lib/pii.js内の正規表現群で、メールアドレス・郵便番号・電話番号・日付・時刻・金額・数量・パスポート番号・法人格(株式会社/Inc./Corp.等)を含む企業名を検出する。マイナンバー(12桁)・クレジットカード番号(13/15/16/19桁、Luhnアルゴリズムで検証)・銀行口座番号(前後に「口座」の語がある7〜8桁)は数字列から判定する。人物名は敬称(様・殿・氏)付きの表記に加え、約140種の代表的な日本人の名字を手がかりに敬称なしの表記も検出する(地名・施設名の一部との誤検出を避ける除外処理あり)。</t>
+        </is>
+      </c>
+      <c r="E5" s="17" t="inlineStr">
         <is>
           <t>実装済み</t>
         </is>
       </c>
     </row>
     <row r="6" ht="42" customHeight="1">
-      <c r="A6" s="9" t="n">
+      <c r="A6" s="17" t="n">
         <v>3</v>
       </c>
-      <c r="B6" s="9" t="inlineStr">
-        <is>
-          <t>複数モデルの切り替え</t>
+      <c r="B6" s="17" t="inlineStr">
+        <is>
+          <t>列見出し/キー名による検出</t>
         </is>
       </c>
       <c r="C6" s="10" t="inlineStr">
         <is>
-          <t>使用するLLMモデルをUI上のセレクトボックスから切り替えられるようにする。</t>
+          <t>表形式データの列見出しやJSONのキー名からカテゴリを機械的に判定する。</t>
         </is>
       </c>
       <c r="D6" s="10" t="inlineStr">
         <is>
-          <t>サーバーの GET /api/models が Ollama の GET /api/tags を呼び出し、ダウンロード済みモデルの一覧を返す。ヘッダーのセレクトボックスに一覧表示し、会話ごとに使用モデルを記憶する。選択したモデル名は POST /api/chat のリクエストに含めて送信し、未指定の場合はサーバーの環境変数 MODEL_NAME が使用される。</t>
-        </is>
-      </c>
-      <c r="E6" s="9" t="inlineStr">
+          <t>xlsx/csvの1行目、pdf内の罫線付き表の1行目を見出しとみなし、「氏名」「電話番号」等のキーワードと一致した列の全セルを該当カテゴリとして検出する。jsonはキー名(例: "phone")から同様に値のカテゴリを判定する。Ollama未接続時でも機能する。</t>
+        </is>
+      </c>
+      <c r="E6" s="17" t="inlineStr">
         <is>
           <t>実装済み</t>
         </is>
       </c>
     </row>
     <row r="7" ht="42" customHeight="1">
-      <c r="A7" s="9" t="n">
+      <c r="A7" s="17" t="n">
         <v>4</v>
       </c>
-      <c r="B7" s="9" t="inlineStr">
-        <is>
-          <t>Dockerによる環境構築</t>
+      <c r="B7" s="17" t="inlineStr">
+        <is>
+          <t>ラベル付きテキストの検出</t>
         </is>
       </c>
       <c r="C7" s="10" t="inlineStr">
         <is>
-          <t>Docker Composeでアプリ本体とOllamaを一括起動できるようにする。</t>
+          <t>自由記述のテキスト中の「ラベル: 値」形式の行を検出する。</t>
         </is>
       </c>
       <c r="D7" s="10" t="inlineStr">
         <is>
-          <t>Dockerfileでアプリ(Node.js 20-alpine)のイメージをビルドし、docker-compose.yml でOllamaコンテナ(ollama/ollama:latest)とアプリコンテナをまとめて起動する。Ollamaのモデルデータは名前付きボリューム ollama_data に永続化する。</t>
-        </is>
-      </c>
-      <c r="E7" s="9" t="inlineStr">
+          <t>pdf/docx/pptx/txt等の自由記述文書で「氏名: 山田太郎」のような「ラベル: 値」形式の行を正規表現で抽出し、ラベルの文言から列見出し検出と同じキーワードでカテゴリを判定する。</t>
+        </is>
+      </c>
+      <c r="E7" s="17" t="inlineStr">
         <is>
           <t>実装済み</t>
         </is>
       </c>
     </row>
     <row r="8" ht="30" customHeight="1">
-      <c r="A8" s="9" t="n">
+      <c r="A8" s="17" t="n">
         <v>5</v>
       </c>
-      <c r="B8" s="9" t="inlineStr">
-        <is>
-          <t>エラーハンドリング</t>
+      <c r="B8" s="17" t="inlineStr">
+        <is>
+          <t>AI(Gemma)による検出</t>
         </is>
       </c>
       <c r="C8" s="10" t="inlineStr">
         <is>
-          <t>Ollama未起動時や通信エラー時に、原因が分かるメッセージを画面に表示する。</t>
+          <t>Ollama経由でGemmaモデルに全15カテゴリの確認を依頼する。</t>
         </is>
       </c>
       <c r="D8" s="10" t="inlineStr">
         <is>
-          <t>サーバーはOllamaへの接続失敗時に502エラーと日本語のエラーメッセージを返却する。フロントエンドはエラーをチャット画面にエラーメッセージとして表示し、送信前の状態に会話履歴を戻す。</t>
-        </is>
-      </c>
-      <c r="E8" s="9" t="inlineStr">
+          <t>抽出テキストをPII_CHUNK_CHAR_LIMIT(既定3000文字)単位に分割し、各チャンクをOllamaのPOST /api/chat(format: "json"、num_predict・temperature:0を指定)に渡す。応答は{"findings":[{"category","text"}]}形式のJSONとしてパースし、他の検出方法の結果とマージする。チャンク数の上限はPII_MAX_CHUNKS(既定40)。Ollama未接続・タイムアウト(既定300秒)の場合は警告を表示し、以降のAI確認を中止して他の検出方法の結果のみを返す。</t>
+        </is>
+      </c>
+      <c r="E8" s="17" t="inlineStr">
         <is>
           <t>実装済み</t>
         </is>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" s="17" t="n">
+        <v>6</v>
+      </c>
+      <c r="B9" s="17" t="inlineStr">
+        <is>
+          <t>検出結果の表示</t>
+        </is>
+      </c>
+      <c r="C9" s="10" t="inlineStr">
+        <is>
+          <t>検出結果をカテゴリ別の色分けバッジと一覧表で表示する。</t>
+        </is>
+      </c>
+      <c r="D9" s="10" t="inlineStr">
+        <is>
+          <t>判定結果を「個人情報なし」「◯件検出」「判定できませんでした」の3状態でバナー表示し、検出された各項目をカテゴリ・検出内容・検出方法(パターン検出/列見出し検出/ラベル検出/AI検出、複数の場合は併記)・場所(シート名/セル番地、ページ番号、行列番号、JSONパス、スライド番号等)の一覧表で表示する。警告(Ollama未接続等)がある場合はその旨を別途表示する。</t>
+        </is>
+      </c>
+      <c r="E9" s="17" t="inlineStr">
+        <is>
+          <t>実装済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="17" t="n">
+        <v>7</v>
+      </c>
+      <c r="B10" s="17" t="inlineStr">
+        <is>
+          <t>利用モデルの固定管理</t>
+        </is>
+      </c>
+      <c r="C10" s="10" t="inlineStr">
+        <is>
+          <t>使用するOllamaモデルをサーバー設定で1つに固定する。</t>
+        </is>
+      </c>
+      <c r="D10" s="10" t="inlineStr">
+        <is>
+          <t>環境変数MODEL_NAME(既定gemma4:e4b)で指定したモデルをアプリ全体で使用する。画面上でのモデル切り替えはできず、ヘッダーに現在のモデル名をバッジ表示する。GET /api/modelsでOllama側に当該モデルが取得済みか確認し、未取得の場合はチェック機能を無効化して警告を表示する。</t>
+        </is>
+      </c>
+      <c r="E10" s="17" t="inlineStr">
+        <is>
+          <t>実装済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="17" t="n">
+        <v>8</v>
+      </c>
+      <c r="B11" s="17" t="inlineStr">
+        <is>
+          <t>アップロード監査ログ</t>
+        </is>
+      </c>
+      <c r="C11" s="10" t="inlineStr">
+        <is>
+          <t>誰が・いつ・何のファイルをチェックしたかをサーバー側に記録する。</t>
+        </is>
+      </c>
+      <c r="D11" s="10" t="inlineStr">
+        <is>
+          <t>アップロードごとにアップロード日時・ログインユーザー名(Google認証時はX-Forwarded-Emailヘッダー、認証なし時はunknown)・ファイル名・拡張子・判定結果の概要(クリーン/検出件数/検出カテゴリ名。検出テキストそのものは含まない)をJSON Lines形式で記録する。環境変数PII_LOG_DIR(既定./logs)配下に1日1ファイル(pii-check-YYYY-MM-DD.log)として、サーバーのローカル時刻(TZ)で日付が変わるタイミングで自動的に分割され、PII_LOG_RETENTION_DAYS(既定90日)より古いファイルは自動削除される。</t>
+        </is>
+      </c>
+      <c r="E11" s="17" t="inlineStr">
+        <is>
+          <t>実装済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="17" t="n">
+        <v>9</v>
+      </c>
+      <c r="B12" s="17" t="inlineStr">
+        <is>
+          <t>Google Workspace認証(SSO)連携(任意・本番構成)</t>
+        </is>
+      </c>
+      <c r="C12" s="10" t="inlineStr">
+        <is>
+          <t>社内向け本番デプロイ時、Google Workspaceアカウントでのログインを必須にする。</t>
+        </is>
+      </c>
+      <c r="D12" s="10" t="inlineStr">
+        <is>
+          <t>oauth2-proxy(docker-compose.prod.yml)をリバースプロキシとして配置し、Google OAuthでログインしたユーザーのうち、環境変数ALLOWED_EMAIL_DOMAINで指定した自社ドメインのアカウントのみ後段のappへのアクセスを許可する。ログイン済みユーザーのメールアドレスはX-Forwarded-Emailヘッダーでappに転送され、アップロード監査ログのユーザー名として利用される。ローカル開発環境(docker-compose.yml単体)では認証なしで利用できる。</t>
+        </is>
+      </c>
+      <c r="E12" s="17" t="inlineStr">
+        <is>
+          <t>実装済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="13"/>
+    <row r="14"/>
+    <row r="15"/>
+    <row r="16"/>
+    <row r="17"/>
+    <row r="18"/>
+    <row r="19"/>
+    <row r="20"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1009,7 +1162,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C14"/>
+  <dimension ref="A1:C30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -1025,209 +1178,241 @@
       </c>
     </row>
     <row r="3" ht="22" customHeight="1">
-      <c r="A3" s="8" t="inlineStr">
+      <c r="A3" s="16" t="inlineStr">
         <is>
           <t>画面/領域</t>
         </is>
       </c>
-      <c r="B3" s="8" t="inlineStr">
+      <c r="B3" s="16" t="inlineStr">
         <is>
           <t>要素</t>
         </is>
       </c>
-      <c r="C3" s="8" t="inlineStr">
+      <c r="C3" s="16" t="inlineStr">
         <is>
           <t>説明</t>
         </is>
       </c>
     </row>
     <row r="4" ht="32" customHeight="1">
-      <c r="A4" s="9" t="inlineStr">
-        <is>
-          <t>チャット画面(全体)</t>
-        </is>
-      </c>
-      <c r="B4" s="9" t="inlineStr">
+      <c r="A4" s="17" t="inlineStr">
+        <is>
+          <t>全体</t>
+        </is>
+      </c>
+      <c r="B4" s="17" t="inlineStr">
         <is>
           <t>レイアウト</t>
         </is>
       </c>
       <c r="C4" s="10" t="inlineStr">
         <is>
-          <t>サイドバー(左)とメインエリア(右)の2カラム構成。1ページのシングルページアプリケーション(public/index.html, app.js, style.css)。</t>
+          <t>グラデーション背景のヒーローヘッダー・紹介カード・アップロードカード・結果表示エリア・フッターで構成される単一ページ(public/index.html, pii.js, style.css)。チャット機能は持たない。</t>
         </is>
       </c>
     </row>
     <row r="5" ht="32" customHeight="1">
-      <c r="A5" s="9" t="inlineStr">
+      <c r="A5" s="17" t="inlineStr">
         <is>
           <t>ヘッダー</t>
         </is>
       </c>
-      <c r="B5" s="9" t="inlineStr">
+      <c r="B5" s="17" t="inlineStr">
         <is>
           <t>アプリ名</t>
         </is>
       </c>
       <c r="C5" s="10" t="inlineStr">
         <is>
-          <t>「Local Gemma Chat」を表示。</t>
+          <t>「個人情報チェック」とサブタイトル「マスキング漏れをローカルLLM(Gemma)でダブルチェック」を表示。</t>
         </is>
       </c>
     </row>
     <row r="6" ht="32" customHeight="1">
-      <c r="A6" s="9" t="inlineStr">
+      <c r="A6" s="17" t="inlineStr">
         <is>
           <t>ヘッダー</t>
         </is>
       </c>
-      <c r="B6" s="9" t="inlineStr">
-        <is>
-          <t>モデル選択(セレクトボックス)</t>
+      <c r="B6" s="17" t="inlineStr">
+        <is>
+          <t>モデルバッジ</t>
         </is>
       </c>
       <c r="C6" s="10" t="inlineStr">
         <is>
-          <t>Ollamaにダウンロード済みのモデル一覧を表示し、選択したモデルを現在の会話に紐付ける。</t>
+          <t>現在使用中のOllamaモデル名を表示。未取得時は「利用不可」と警告色で表示し、チェック機能を無効化する。</t>
         </is>
       </c>
     </row>
     <row r="7" ht="32" customHeight="1">
-      <c r="A7" s="9" t="inlineStr">
-        <is>
-          <t>サイドバー</t>
-        </is>
-      </c>
-      <c r="B7" s="9" t="inlineStr">
-        <is>
-          <t>新規チャットボタン</t>
+      <c r="A7" s="17" t="inlineStr">
+        <is>
+          <t>紹介カード</t>
+        </is>
+      </c>
+      <c r="B7" s="17" t="inlineStr">
+        <is>
+          <t>説明文</t>
         </is>
       </c>
       <c r="C7" s="10" t="inlineStr">
         <is>
-          <t>「+ 新しいチャット」ボタン押下で空の会話を作成し、一覧の先頭に追加する。</t>
+          <t>対応ファイル形式とチェック方法の概要を表示。</t>
         </is>
       </c>
     </row>
     <row r="8" ht="32" customHeight="1">
-      <c r="A8" s="9" t="inlineStr">
-        <is>
-          <t>サイドバー</t>
-        </is>
-      </c>
-      <c r="B8" s="9" t="inlineStr">
-        <is>
-          <t>会話一覧</t>
+      <c r="A8" s="17" t="inlineStr">
+        <is>
+          <t>紹介カード</t>
+        </is>
+      </c>
+      <c r="B8" s="17" t="inlineStr">
+        <is>
+          <t>カテゴリチップ</t>
         </is>
       </c>
       <c r="C8" s="10" t="inlineStr">
         <is>
-          <t>保存済みの会話をタイトルで一覧表示。クリックで会話を切り替える。選択中の会話はハイライト表示される。</t>
+          <t>検出対象の15カテゴリをカテゴリごとの色分けチップで一覧表示。</t>
         </is>
       </c>
     </row>
     <row r="9" ht="32" customHeight="1">
-      <c r="A9" s="9" t="inlineStr">
-        <is>
-          <t>サイドバー</t>
-        </is>
-      </c>
-      <c r="B9" s="9" t="inlineStr">
-        <is>
-          <t>会話の削除</t>
+      <c r="A9" s="17" t="inlineStr">
+        <is>
+          <t>アップロードカード</t>
+        </is>
+      </c>
+      <c r="B9" s="17" t="inlineStr">
+        <is>
+          <t>ドロップゾーン</t>
         </is>
       </c>
       <c r="C9" s="10" t="inlineStr">
         <is>
-          <t>各会話項目にホバーすると削除ボタン(✕)が表示され、クリックで該当会話を削除する。</t>
+          <t>ファイルをドラッグ&amp;ドロップ、またはクリックして選択(.xlsx/.pdf/.docx/.pptx/.csv/.txt/.json、最大50MB)。選択中のファイル名を表示。</t>
         </is>
       </c>
     </row>
     <row r="10" ht="32" customHeight="1">
-      <c r="A10" s="9" t="inlineStr">
-        <is>
-          <t>メインエリア(チャットログ)</t>
-        </is>
-      </c>
-      <c r="B10" s="9" t="inlineStr">
-        <is>
-          <t>ユーザー発言</t>
+      <c r="A10" s="17" t="inlineStr">
+        <is>
+          <t>アップロードカード</t>
+        </is>
+      </c>
+      <c r="B10" s="17" t="inlineStr">
+        <is>
+          <t>チェックするボタン</t>
         </is>
       </c>
       <c r="C10" s="10" t="inlineStr">
         <is>
-          <t>吹き出しを画面右寄せ・青背景・白文字で表示する。</t>
+          <t>クリックでPOST /api/pii-checkを実行する。処理中はスピナーを表示し、ボタンを非活性化する。</t>
         </is>
       </c>
     </row>
     <row r="11" ht="32" customHeight="1">
-      <c r="A11" s="9" t="inlineStr">
-        <is>
-          <t>メインエリア(チャットログ)</t>
-        </is>
-      </c>
-      <c r="B11" s="9" t="inlineStr">
-        <is>
-          <t>アシスタント発言</t>
+      <c r="A11" s="17" t="inlineStr">
+        <is>
+          <t>アップロードカード</t>
+        </is>
+      </c>
+      <c r="B11" s="17" t="inlineStr">
+        <is>
+          <t>注意書き</t>
         </is>
       </c>
       <c r="C11" s="10" t="inlineStr">
         <is>
-          <t>吹き出しを画面左寄せ・グレー背景で表示し、ストリーミングで受信するたびにテキストを追記表示する。</t>
+          <t>「このチェックは補助的なものであり、結果によらず目視でも必ず確認してください」という注意文を表示。</t>
         </is>
       </c>
     </row>
     <row r="12" ht="32" customHeight="1">
-      <c r="A12" s="9" t="inlineStr">
-        <is>
-          <t>メインエリア(チャットログ)</t>
-        </is>
-      </c>
-      <c r="B12" s="9" t="inlineStr">
-        <is>
-          <t>エラーメッセージ</t>
+      <c r="A12" s="17" t="inlineStr">
+        <is>
+          <t>結果表示エリア</t>
+        </is>
+      </c>
+      <c r="B12" s="17" t="inlineStr">
+        <is>
+          <t>サマリーバナー</t>
         </is>
       </c>
       <c r="C12" s="10" t="inlineStr">
         <is>
-          <t>通信エラー等が発生した場合、中央揃え・赤文字でエラー内容を表示する。</t>
+          <t>「個人情報なし(緑)」「◯件検出(赤)」「判定できませんでした(黄/警告)」のいずれかを色分け表示。</t>
         </is>
       </c>
     </row>
     <row r="13" ht="32" customHeight="1">
-      <c r="A13" s="9" t="inlineStr">
-        <is>
-          <t>フッター(入力欄)</t>
-        </is>
-      </c>
-      <c r="B13" s="9" t="inlineStr">
-        <is>
-          <t>テキストエリア</t>
+      <c r="A13" s="17" t="inlineStr">
+        <is>
+          <t>結果表示エリア</t>
+        </is>
+      </c>
+      <c r="B13" s="17" t="inlineStr">
+        <is>
+          <t>警告一覧</t>
         </is>
       </c>
       <c r="C13" s="10" t="inlineStr">
         <is>
-          <t>複数行入力可能な自動リサイズのテキストエリア。Enterで送信、Shift+Enterで改行。</t>
+          <t>Ollama未接続・タイムアウト・AI解析失敗等の警告メッセージを箇条書きで表示。</t>
         </is>
       </c>
     </row>
     <row r="14" ht="32" customHeight="1">
-      <c r="A14" s="9" t="inlineStr">
-        <is>
-          <t>フッター(入力欄)</t>
-        </is>
-      </c>
-      <c r="B14" s="9" t="inlineStr">
-        <is>
-          <t>送信ボタン</t>
+      <c r="A14" s="17" t="inlineStr">
+        <is>
+          <t>結果表示エリア</t>
+        </is>
+      </c>
+      <c r="B14" s="17" t="inlineStr">
+        <is>
+          <t>検出結果テーブル</t>
         </is>
       </c>
       <c r="C14" s="10" t="inlineStr">
         <is>
-          <t>クリックまたはEnterキーでメッセージを送信する。応答待機中は非活性化される。</t>
-        </is>
-      </c>
-    </row>
+          <t>カテゴリ(色分けバッジ)・検出内容・検出方法・場所の列を持つ一覧表を表示。</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="17" t="inlineStr">
+        <is>
+          <t>フッター</t>
+        </is>
+      </c>
+      <c r="B15" s="17" t="inlineStr">
+        <is>
+          <t>注意書き</t>
+        </is>
+      </c>
+      <c r="C15" s="10" t="inlineStr">
+        <is>
+          <t>ファイル内容・検出された個人情報の中身は保存されないこと、監査のためアップロード日時・ユーザー名・ファイル名・判定結果の概要のみサーバーに記録されることを明示。</t>
+        </is>
+      </c>
+    </row>
+    <row r="16"/>
+    <row r="17"/>
+    <row r="18"/>
+    <row r="19"/>
+    <row r="20"/>
+    <row r="21"/>
+    <row r="22"/>
+    <row r="23"/>
+    <row r="24"/>
+    <row r="25"/>
+    <row r="26"/>
+    <row r="27"/>
+    <row r="28"/>
+    <row r="29"/>
+    <row r="30"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1239,7 +1424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:E20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1257,39 +1442,39 @@
       </c>
     </row>
     <row r="3" ht="22" customHeight="1">
-      <c r="A3" s="8" t="inlineStr">
+      <c r="A3" s="16" t="inlineStr">
         <is>
           <t>メソッド</t>
         </is>
       </c>
-      <c r="B3" s="8" t="inlineStr">
+      <c r="B3" s="16" t="inlineStr">
         <is>
           <t>パス</t>
         </is>
       </c>
-      <c r="C3" s="8" t="inlineStr">
+      <c r="C3" s="16" t="inlineStr">
         <is>
           <t>リクエスト</t>
         </is>
       </c>
-      <c r="D3" s="8" t="inlineStr">
+      <c r="D3" s="16" t="inlineStr">
         <is>
           <t>レスポンス</t>
         </is>
       </c>
-      <c r="E3" s="8" t="inlineStr">
+      <c r="E3" s="16" t="inlineStr">
         <is>
           <t>説明</t>
         </is>
       </c>
     </row>
     <row r="4" ht="24" customHeight="1">
-      <c r="A4" s="9" t="inlineStr">
+      <c r="A4" s="17" t="inlineStr">
         <is>
           <t>GET</t>
         </is>
       </c>
-      <c r="B4" s="9" t="inlineStr">
+      <c r="B4" s="17" t="inlineStr">
         <is>
           <t>/ (および静的ファイル)</t>
         </is>
@@ -1301,7 +1486,7 @@
       </c>
       <c r="D4" s="10" t="inlineStr">
         <is>
-          <t>public/ 配下の静的ファイル(index.html, app.js, style.css)</t>
+          <t>public/配下の静的ファイル(index.html, pii.js, style.css)</t>
         </is>
       </c>
       <c r="E4" s="10" t="inlineStr">
@@ -1311,12 +1496,12 @@
       </c>
     </row>
     <row r="5" ht="70" customHeight="1">
-      <c r="A5" s="9" t="inlineStr">
+      <c r="A5" s="17" t="inlineStr">
         <is>
           <t>GET</t>
         </is>
       </c>
-      <c r="B5" s="9" t="inlineStr">
+      <c r="B5" s="17" t="inlineStr">
         <is>
           <t>/api/models</t>
         </is>
@@ -1329,44 +1514,83 @@
       <c r="D5" s="10" t="inlineStr">
         <is>
           <t>200: { models: string[], default: string }
-(Ollama未起動時は models: [] を返す)</t>
+(Ollama未起動時はmodels: [])</t>
         </is>
       </c>
       <c r="E5" s="10" t="inlineStr">
         <is>
-          <t>Ollamaの GET /api/tags を呼び出し、ダウンロード済みモデル名の一覧と既定モデル名(環境変数 MODEL_NAME)を返す。</t>
+          <t>Ollamaの GET /api/tags を呼び出し、取得済みモデル名の一覧と既定モデル名(環境変数MODEL_NAME)を返す。フロントエンドはdefaultがmodelsに含まれるかでチェック機能の有効/無効を判定する。</t>
         </is>
       </c>
     </row>
     <row r="6" ht="70" customHeight="1">
-      <c r="A6" s="9" t="inlineStr">
+      <c r="A6" s="17" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="B6" s="17" t="inlineStr">
+        <is>
+          <t>/api/pii-categories</t>
+        </is>
+      </c>
+      <c r="C6" s="10" t="inlineStr">
+        <is>
+          <t>なし</t>
+        </is>
+      </c>
+      <c r="D6" s="10" t="inlineStr">
+        <is>
+          <t>200: { categories: { key, label, method }[] }</t>
+        </is>
+      </c>
+      <c r="E6" s="10" t="inlineStr">
+        <is>
+          <t>検出対象の15カテゴリの一覧(キー・日本語ラベル・検出方法)を返す。画面のカテゴリチップ・結果テーブルの表示に使用する。</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="17" t="inlineStr">
         <is>
           <t>POST</t>
         </is>
       </c>
-      <c r="B6" s="9" t="inlineStr">
-        <is>
-          <t>/api/chat</t>
-        </is>
-      </c>
-      <c r="C6" s="10" t="inlineStr">
-        <is>
-          <t>{ messages: { role: "user"|"assistant", content: string }[], model?: string }</t>
-        </is>
-      </c>
-      <c r="D6" s="10" t="inlineStr">
-        <is>
-          <t>200: text/plain(chunked)でストリーミングされる生成テキスト
-400: { error }(messages不正)
-502: { error }(Ollama未起動/エラー時)</t>
-        </is>
-      </c>
-      <c r="E6" s="10" t="inlineStr">
-        <is>
-          <t>Ollamaの POST /api/chat ( stream: true ) にリクエストを転送する。model省略時は環境変数 MODEL_NAME を使用。Ollamaから返るNDJSONストリームを1行ずつ解析し、message.content のみを抽出してチャンク単位でクライアントへ返す。</t>
-        </is>
-      </c>
-    </row>
+      <c r="B7" s="17" t="inlineStr">
+        <is>
+          <t>/api/pii-check</t>
+        </is>
+      </c>
+      <c r="C7" s="10" t="inlineStr">
+        <is>
+          <t>multipart/form-data: file(アップロードファイル、最大50MB)</t>
+        </is>
+      </c>
+      <c r="D7" s="10" t="inlineStr">
+        <is>
+          <t>200: { fileName, model, isClean, extractionFailed?, findings: { category, text, sources, locations }[], warnings: string[], categories }
+400: { error }(ファイル未指定・非対応形式・サイズ超過・解析失敗時)</t>
+        </is>
+      </c>
+      <c r="E7" s="10" t="inlineStr">
+        <is>
+          <t>アップロードファイルからテキストを抽出し、正規表現・列見出し/キー名・ラベル・AI(Ollama経由のGemma)の4方式で個人情報を検出してマージした結果を返す。処理結果はアップロード監査ログに記録される(「5. データ保存・監査ログ仕様」参照)。</t>
+        </is>
+      </c>
+    </row>
+    <row r="8"/>
+    <row r="9"/>
+    <row r="10"/>
+    <row r="11"/>
+    <row r="12"/>
+    <row r="13"/>
+    <row r="14"/>
+    <row r="15"/>
+    <row r="16"/>
+    <row r="17"/>
+    <row r="18"/>
+    <row r="19"/>
+    <row r="20"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1378,7 +1602,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B7"/>
+  <dimension ref="A1:B20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1388,76 +1612,107 @@
     <row r="1">
       <c r="A1" s="11" t="inlineStr">
         <is>
-          <t>5. データ保存仕様(会話履歴)</t>
+          <t>5. データ保存・監査ログ仕様</t>
         </is>
       </c>
     </row>
     <row r="3" ht="20" customHeight="1">
-      <c r="A3" s="12" t="inlineStr">
-        <is>
-          <t>保存先</t>
+      <c r="A3" s="15" t="inlineStr">
+        <is>
+          <t>アップロードファイル・検出結果</t>
         </is>
       </c>
       <c r="B3" s="13" t="inlineStr">
         <is>
-          <t>ブラウザの localStorage(サーバーやファイルには保存されない)。</t>
+          <t>処理はすべてサーバーのメモリ上で行われ、アップロードされたファイルの内容や検出された個人情報の中身はディスク・サーバーのいずれにも保存されない。</t>
         </is>
       </c>
     </row>
     <row r="4" ht="20" customHeight="1">
-      <c r="A4" s="12" t="inlineStr">
-        <is>
-          <t>キー: gemma-chat-conversations</t>
+      <c r="A4" s="15" t="inlineStr">
+        <is>
+          <t>アップロード監査ログの保存先</t>
         </is>
       </c>
       <c r="B4" s="13" t="inlineStr">
         <is>
-          <t>会話一覧を表すJSON配列。ページ読み込み時に読み込まれ、更新の都度上書き保存される。</t>
+          <t>環境変数PII_LOG_DIR(既定./logs。Docker利用時は/app/logs、名前付きボリュームpii_logsで永続化)配下にJSON Lines形式で記録される(lib/auditLog.js、winston / winston-daily-rotate-fileを使用)。</t>
         </is>
       </c>
     </row>
     <row r="5" ht="20" customHeight="1">
-      <c r="A5" s="12" t="inlineStr">
-        <is>
-          <t>キー: gemma-chat-current-id</t>
+      <c r="A5" s="15" t="inlineStr">
+        <is>
+          <t>ログファイルの分割</t>
         </is>
       </c>
       <c r="B5" s="13" t="inlineStr">
         <is>
-          <t>現在表示中の会話ID(文字列)。</t>
+          <t>1日1ファイル(ファイル名: pii-check-YYYY-MM-DD.log)。サーバーのローカル時刻(環境変数TZ、既定Asia/Tokyo)で日付が変わるタイミングで自動的に新しいファイルに切り替わる。</t>
         </is>
       </c>
     </row>
     <row r="6" ht="80" customHeight="1">
-      <c r="A6" s="12" t="inlineStr">
-        <is>
-          <t>会話オブジェクトの構造</t>
+      <c r="A6" s="15" t="inlineStr">
+        <is>
+          <t>保持期間</t>
         </is>
       </c>
       <c r="B6" s="13" t="inlineStr">
         <is>
-          <t>id: 会話を一意に識別するUUID
-title: 会話タイトル(先頭のユーザー発言から自動生成、最大30文字)
-model: この会話で使用するOllamaモデル名
-messages: { role: "user"|"assistant", content: string } の配列(会話全文)
-updatedAt: 最終更新日時(UNIXミリ秒)</t>
+          <t>環境変数PII_LOG_RETENTION_DAYS(既定90日)より古いログファイルは自動的に削除される。</t>
         </is>
       </c>
     </row>
     <row r="7" ht="48" customHeight="1">
-      <c r="A7" s="12" t="inlineStr">
+      <c r="A7" s="15" t="inlineStr">
+        <is>
+          <t>ログ1件の記録項目</t>
+        </is>
+      </c>
+      <c r="B7" s="13" t="inlineStr">
+        <is>
+          <t>uploadedAt(アップロード日時)/ user(ログインユーザー名)/ fileName(ファイル名)/ fileType(拡張子)/ status(checked・extraction_failed・parse_errorのいずれか)/ isClean(個人情報が検出されなかったか、checked時のみ)/ findingsCount(検出件数、checked時のみ)/ categories(検出されたカテゴリ名の一覧、checked時のみ。検出テキストそのものは含まない)。</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="15" t="inlineStr">
+        <is>
+          <t>ログインユーザー名の取得方法</t>
+        </is>
+      </c>
+      <c r="B8" s="13" t="inlineStr">
+        <is>
+          <t>Google認証(oauth2-proxy)経由でアクセスした場合、oauth2-proxyが付与するX-Forwarded-Emailヘッダーからログイン中のGoogleアカウントのメールアドレスを取得する。認証なしでアクセスできる構成では取得できないためunknownとなる。appコンテナに直接到達できない構成(docker-compose.prod.yml/auth-test.yml)でのみこのヘッダーは信頼できる(直接到達できる構成ではクライアントが任意の値を送信できるため、ユーザー名は参考情報となる)。</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="15" t="inlineStr">
         <is>
           <t>留意事項</t>
         </is>
       </c>
-      <c r="B7" s="13" t="inlineStr">
-        <is>
-          <t>・ブラウザのデータ消去(キャッシュクリア等)で履歴も失われる。
-・別ブラウザ/別端末間で履歴は共有されない。
-・複数ユーザーでの共有を要する場合はサーバーサイドでの永続化(DB等)が別途必要(「7. 今後の課題」参照)。</t>
-        </is>
-      </c>
-    </row>
+      <c r="B9" s="13" t="inlineStr">
+        <is>
+          <t>・ログファイル自体にも検出された個人情報の中身(氏名・電話番号等の実際の値)は一切記録されない。
+・複数レプリカで運用する場合、ログはPodごとのローカルボリュームに分散して記録される(現状はreplicas: 1を想定)。
+・監査ログの消去・改ざん対策(読み取り専用化、外部ログ基盤への転送等)は現状実装していない。</t>
+        </is>
+      </c>
+    </row>
+    <row r="10"/>
+    <row r="11"/>
+    <row r="12"/>
+    <row r="13"/>
+    <row r="14"/>
+    <row r="15"/>
+    <row r="16"/>
+    <row r="17"/>
+    <row r="18"/>
+    <row r="19"/>
+    <row r="20"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1469,7 +1724,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C21"/>
+  <dimension ref="A1:C60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1494,11 +1749,12 @@
     <row r="4" ht="60" customHeight="1">
       <c r="A4" s="14" t="inlineStr">
         <is>
-          <t>ブラウザ ⇔ Node.js/Expressサーバー(ポート3000、コンテナ名 app) ⇔ Ollamaサーバー(ポート11434、コンテナ名 ollama)
-ブラウザはExpressサーバーとのみ通信し、Ollamaへのアクセスはすべてサーバー経由(プロキシ)で行う。Docker利用時、appコンテナは環境変数 OLLAMA_HOST=http://ollama:11434 でOllamaコンテナに接続する。</t>
-        </is>
-      </c>
-    </row>
+          <t>ブラウザ ⇔ (本番構成の場合) oauth2-proxy(Google Workspace認証、ポート443/4180) ⇔ Node.js/Expressサーバー(ポート3000、コンテナ名app) ⇔ Ollamaサーバー(ポート11434、コンテナ名ollama)
+ブラウザはExpressサーバー(または手前のoauth2-proxy)とのみ通信し、Ollamaへのアクセスはすべてサーバー経由(プロキシ)で行う。Docker利用時、appコンテナは環境変数OLLAMA_HOST=http://ollama:11434でOllamaコンテナに接続する。ローカル開発用のdocker-compose.ymlは認証なし構成、docker-compose.prod.ymlは社内ネットワーク/VPN限定+Google Workspace SSO構成、docker-compose.auth-test.ymlはGoogle認証のローカル動作確認用オーバーレイ。</t>
+        </is>
+      </c>
+    </row>
+    <row r="5"/>
     <row r="6">
       <c r="A6" s="7" t="inlineStr">
         <is>
@@ -1507,216 +1763,529 @@
       </c>
     </row>
     <row r="7" ht="22" customHeight="1">
-      <c r="A7" s="8" t="inlineStr">
+      <c r="A7" s="16" t="inlineStr">
         <is>
           <t>区分</t>
         </is>
       </c>
-      <c r="B7" s="8" t="inlineStr">
+      <c r="B7" s="16" t="inlineStr">
         <is>
           <t>技術/製品</t>
         </is>
       </c>
-      <c r="C7" s="8" t="inlineStr">
+      <c r="C7" s="16" t="inlineStr">
         <is>
           <t>バージョン・備考</t>
         </is>
       </c>
     </row>
     <row r="8" ht="26" customHeight="1">
-      <c r="A8" s="9" t="inlineStr">
+      <c r="A8" s="17" t="inlineStr">
         <is>
           <t>フロントエンド</t>
         </is>
       </c>
-      <c r="B8" s="9" t="inlineStr">
+      <c r="B8" s="17" t="inlineStr">
         <is>
           <t>HTML / CSS / JavaScript</t>
         </is>
       </c>
       <c r="C8" s="10" t="inlineStr">
         <is>
-          <t>フレームワーク不使用(素のJS)。public/ 配下に配置。</t>
+          <t>フレームワーク不使用(素のJS)。public/配下に配置。</t>
         </is>
       </c>
     </row>
     <row r="9" ht="26" customHeight="1">
-      <c r="A9" s="9" t="inlineStr">
+      <c r="A9" s="17" t="inlineStr">
         <is>
           <t>バックエンド</t>
         </is>
       </c>
-      <c r="B9" s="9" t="inlineStr">
+      <c r="B9" s="17" t="inlineStr">
         <is>
           <t>Node.js</t>
         </is>
       </c>
       <c r="C9" s="10" t="inlineStr">
         <is>
-          <t>18以上(Dockerイメージは node:20-alpine)</t>
+          <t>18以上(Dockerイメージはnode:20-alpine)</t>
         </is>
       </c>
     </row>
     <row r="10" ht="26" customHeight="1">
-      <c r="A10" s="9" t="inlineStr">
+      <c r="A10" s="17" t="inlineStr">
         <is>
           <t>バックエンド</t>
         </is>
       </c>
-      <c r="B10" s="9" t="inlineStr">
+      <c r="B10" s="17" t="inlineStr">
         <is>
           <t>Express</t>
         </is>
       </c>
       <c r="C10" s="10" t="inlineStr">
         <is>
-          <t>^4.19.2(server.js でAPIサーバーを実装)</t>
+          <t>^4.19.2(server.jsでAPIサーバーを実装)</t>
         </is>
       </c>
     </row>
     <row r="11" ht="26" customHeight="1">
-      <c r="A11" s="9" t="inlineStr">
+      <c r="A11" s="17" t="inlineStr">
+        <is>
+          <t>バックエンド</t>
+        </is>
+      </c>
+      <c r="B11" s="17" t="inlineStr">
+        <is>
+          <t>multer</t>
+        </is>
+      </c>
+      <c r="C11" s="10" t="inlineStr">
+        <is>
+          <t>^2.3.0(ファイルアップロード受付、メモリストレージ、最大50MB)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="26" customHeight="1">
+      <c r="A12" s="17" t="inlineStr">
+        <is>
+          <t>ファイル解析</t>
+        </is>
+      </c>
+      <c r="B12" s="17" t="inlineStr">
+        <is>
+          <t>exceljs</t>
+        </is>
+      </c>
+      <c r="C12" s="10" t="inlineStr">
+        <is>
+          <t>^4.4.0(.xlsx解析)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="26" customHeight="1">
+      <c r="A13" s="17" t="inlineStr">
+        <is>
+          <t>ファイル解析</t>
+        </is>
+      </c>
+      <c r="B13" s="17" t="inlineStr">
+        <is>
+          <t>pdf-parse</t>
+        </is>
+      </c>
+      <c r="C13" s="10" t="inlineStr">
+        <is>
+          <t>^2.4.5(.pdf解析・表構造検出)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="26" customHeight="1">
+      <c r="A14" s="17" t="inlineStr">
+        <is>
+          <t>ファイル解析</t>
+        </is>
+      </c>
+      <c r="B14" s="17" t="inlineStr">
+        <is>
+          <t>mammoth</t>
+        </is>
+      </c>
+      <c r="C14" s="10" t="inlineStr">
+        <is>
+          <t>^1.13.0(.docx解析)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="17" t="inlineStr">
+        <is>
+          <t>ファイル解析</t>
+        </is>
+      </c>
+      <c r="B15" s="17" t="inlineStr">
+        <is>
+          <t>jszip</t>
+        </is>
+      </c>
+      <c r="C15" s="10" t="inlineStr">
+        <is>
+          <t>^3.10.2(.pptx・zip内XML解析)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="17" t="inlineStr">
+        <is>
+          <t>ファイル解析</t>
+        </is>
+      </c>
+      <c r="B16" s="17" t="inlineStr">
+        <is>
+          <t>csv-parse</t>
+        </is>
+      </c>
+      <c r="C16" s="10" t="inlineStr">
+        <is>
+          <t>^7.0.3(.csv解析)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="17" t="inlineStr">
+        <is>
+          <t>ファイル解析</t>
+        </is>
+      </c>
+      <c r="B17" s="17" t="inlineStr">
+        <is>
+          <t>iconv-lite</t>
+        </is>
+      </c>
+      <c r="C17" s="10" t="inlineStr">
+        <is>
+          <t>^0.7.3(.txt/.csv/.jsonの文字コード自動判定・変換、Shift_JIS対応)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="22" customHeight="1">
+      <c r="A18" s="18" t="inlineStr">
+        <is>
+          <t>監査ログ</t>
+        </is>
+      </c>
+      <c r="B18" s="18" t="inlineStr">
+        <is>
+          <t>winston / winston-daily-rotate-file</t>
+        </is>
+      </c>
+      <c r="C18" s="19" t="inlineStr">
+        <is>
+          <t>^3.19.0 / ^5.0.0(日次ローテーション・保持日数管理)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="26" customHeight="1">
+      <c r="A19" s="17" t="inlineStr">
         <is>
           <t>LLM実行基盤</t>
         </is>
       </c>
-      <c r="B11" s="9" t="inlineStr">
+      <c r="B19" s="17" t="inlineStr">
         <is>
           <t>Ollama</t>
         </is>
       </c>
-      <c r="C11" s="10" t="inlineStr">
+      <c r="C19" s="10" t="inlineStr">
         <is>
           <t>ローカルまたはDockerコンテナ(ollama/ollama:latest)で稼働。</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="26" customHeight="1">
-      <c r="A12" s="9" t="inlineStr">
+    <row r="20" ht="26" customHeight="1">
+      <c r="A20" s="17" t="inlineStr">
         <is>
           <t>使用モデル</t>
         </is>
       </c>
-      <c r="B12" s="9" t="inlineStr">
-        <is>
-          <t>Gemma</t>
-        </is>
-      </c>
-      <c r="C12" s="10" t="inlineStr">
-        <is>
-          <t>既定タグ: gemma4(存在しない場合は gemma3 等に読み替え)</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="26" customHeight="1">
-      <c r="A13" s="9" t="inlineStr">
+      <c r="B20" s="17" t="inlineStr">
+        <is>
+          <t>Gemma 4</t>
+        </is>
+      </c>
+      <c r="C20" s="10" t="inlineStr">
+        <is>
+          <t>既定タグ: gemma4:e4b(アプリ全体で1モデルに固定、MODEL_NAMEで変更可)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="26" customHeight="1">
+      <c r="A21" s="17" t="inlineStr">
+        <is>
+          <t>認証(本番構成・任意)</t>
+        </is>
+      </c>
+      <c r="B21" s="17" t="inlineStr">
+        <is>
+          <t>oauth2-proxy</t>
+        </is>
+      </c>
+      <c r="C21" s="10" t="inlineStr">
+        <is>
+          <t>quay.io/oauth2-proxy/oauth2-proxy:latest(Google Workspace OIDC)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="17" t="inlineStr">
         <is>
           <t>コンテナ</t>
         </is>
       </c>
-      <c r="B13" s="9" t="inlineStr">
+      <c r="B22" s="17" t="inlineStr">
         <is>
           <t>Docker / Docker Compose</t>
         </is>
       </c>
-      <c r="C13" s="10" t="inlineStr">
-        <is>
-          <t>Dockerfile と docker-compose.yml を用意。</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="26" customHeight="1">
-      <c r="A14" s="9" t="inlineStr">
+      <c r="C22" s="10" t="inlineStr">
+        <is>
+          <t>Dockerfileとdocker-compose.yml(開発用)/docker-compose.prod.yml(本番)/docker-compose.auth-test.yml(認証確認用)を用意。</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="17" t="inlineStr">
+        <is>
+          <t>オーケストレーション(任意)</t>
+        </is>
+      </c>
+      <c r="B23" s="17" t="inlineStr">
+        <is>
+          <t>Kubernetes</t>
+        </is>
+      </c>
+      <c r="C23" s="10" t="inlineStr">
+        <is>
+          <t>k8s/配下のマニフェストで既存クラスタへkubectlデプロイ可能(DEPLOY_K8S.md参照)。</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="17" t="inlineStr">
         <is>
           <t>データ永続化</t>
         </is>
       </c>
-      <c r="B14" s="9" t="inlineStr">
+      <c r="B24" s="17" t="inlineStr">
         <is>
           <t>Dockerボリューム</t>
         </is>
       </c>
-      <c r="C14" s="10" t="inlineStr">
-        <is>
-          <t>ollama_data にOllamaのモデルデータを永続化。</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="7" t="inlineStr">
+      <c r="C24" s="10" t="inlineStr">
+        <is>
+          <t>ollama_data(モデルデータ)、pii_logs(アップロード監査ログ)を永続化。</t>
+        </is>
+      </c>
+    </row>
+    <row r="25"/>
+    <row r="26">
+      <c r="A26" s="7" t="inlineStr">
         <is>
           <t>環境変数</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="22" customHeight="1">
-      <c r="A18" s="8" t="inlineStr">
+    <row r="27">
+      <c r="A27" s="16" t="inlineStr">
         <is>
           <t>変数名</t>
         </is>
       </c>
-      <c r="B18" s="8" t="inlineStr">
+      <c r="B27" s="16" t="inlineStr">
         <is>
           <t>既定値</t>
         </is>
       </c>
-      <c r="C18" s="8" t="inlineStr">
+      <c r="C27" s="16" t="inlineStr">
         <is>
           <t>説明</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="26" customHeight="1">
-      <c r="A19" s="9" t="inlineStr">
+    <row r="28">
+      <c r="A28" s="17" t="inlineStr">
         <is>
           <t>PORT</t>
         </is>
       </c>
-      <c r="B19" s="9" t="inlineStr">
+      <c r="B28" s="17" t="inlineStr">
         <is>
           <t>3000</t>
         </is>
       </c>
-      <c r="C19" s="10" t="inlineStr">
+      <c r="C28" s="10" t="inlineStr">
         <is>
           <t>Webアプリ(Expressサーバー)の待受ポート。</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="26" customHeight="1">
-      <c r="A20" s="9" t="inlineStr">
+    <row r="29">
+      <c r="A29" s="17" t="inlineStr">
         <is>
           <t>OLLAMA_HOST</t>
         </is>
       </c>
-      <c r="B20" s="9" t="inlineStr">
+      <c r="B29" s="17" t="inlineStr">
         <is>
           <t>http://127.0.0.1:11434</t>
         </is>
       </c>
-      <c r="C20" s="10" t="inlineStr">
-        <is>
-          <t>Ollamaサーバーのアドレス。Docker利用時は http://ollama:11434 を指定。</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="26" customHeight="1">
-      <c r="A21" s="9" t="inlineStr">
+      <c r="C29" s="10" t="inlineStr">
+        <is>
+          <t>Ollamaサーバーのアドレス。Docker利用時はhttp://ollama:11434を指定。</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="17" t="inlineStr">
         <is>
           <t>MODEL_NAME</t>
         </is>
       </c>
-      <c r="B21" s="9" t="inlineStr">
-        <is>
-          <t>gemma4</t>
-        </is>
-      </c>
-      <c r="C21" s="10" t="inlineStr">
-        <is>
-          <t>既定で使用するOllamaのモデル名/タグ。POST /api/chat で model 未指定時に使用。</t>
-        </is>
-      </c>
-    </row>
+      <c r="B30" s="17" t="inlineStr">
+        <is>
+          <t>gemma4:e4b</t>
+        </is>
+      </c>
+      <c r="C30" s="10" t="inlineStr">
+        <is>
+          <t>使用するOllamaモデル名/タグ。アプリ全体で1つに固定(画面上での切替不可)。</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="17" t="inlineStr">
+        <is>
+          <t>OLLAMA_TIMEOUT_MS</t>
+        </is>
+      </c>
+      <c r="B31" s="17" t="inlineStr">
+        <is>
+          <t>300000(5分)</t>
+        </is>
+      </c>
+      <c r="C31" s="10" t="inlineStr">
+        <is>
+          <t>個人情報チェックでOllamaの応答を待つ上限時間。</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="17" t="inlineStr">
+        <is>
+          <t>OLLAMA_NUM_PREDICT</t>
+        </is>
+      </c>
+      <c r="B32" s="17" t="inlineStr">
+        <is>
+          <t>500</t>
+        </is>
+      </c>
+      <c r="C32" s="10" t="inlineStr">
+        <is>
+          <t>AI検出1回あたりの最大生成トークン数。</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="17" t="inlineStr">
+        <is>
+          <t>PII_CHUNK_CHAR_LIMIT</t>
+        </is>
+      </c>
+      <c r="B33" s="17" t="inlineStr">
+        <is>
+          <t>3000</t>
+        </is>
+      </c>
+      <c r="C33" s="10" t="inlineStr">
+        <is>
+          <t>AIに1回に渡すテキストの最大文字数。</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="17" t="inlineStr">
+        <is>
+          <t>PII_MAX_CHUNKS</t>
+        </is>
+      </c>
+      <c r="B34" s="17" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="C34" s="10" t="inlineStr">
+        <is>
+          <t>AIに渡すチャンク数の上限(超過分は正規表現等のみで判定)。</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="17" t="inlineStr">
+        <is>
+          <t>PII_LOG_DIR</t>
+        </is>
+      </c>
+      <c r="B35" s="17" t="inlineStr">
+        <is>
+          <t>./logs</t>
+        </is>
+      </c>
+      <c r="C35" s="10" t="inlineStr">
+        <is>
+          <t>アップロード監査ログの保存先ディレクトリ。</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="17" t="inlineStr">
+        <is>
+          <t>PII_LOG_RETENTION_DAYS</t>
+        </is>
+      </c>
+      <c r="B36" s="17" t="inlineStr">
+        <is>
+          <t>90</t>
+        </is>
+      </c>
+      <c r="C36" s="10" t="inlineStr">
+        <is>
+          <t>アップロード監査ログの保持日数(これより古いファイルは自動削除)。</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="17" t="inlineStr">
+        <is>
+          <t>TZ</t>
+        </is>
+      </c>
+      <c r="B37" s="17" t="inlineStr">
+        <is>
+          <t>(システム既定)</t>
+        </is>
+      </c>
+      <c r="C37" s="10" t="inlineStr">
+        <is>
+          <t>ログの日付区切りに使うタイムゾーン(例: Asia/Tokyo)。</t>
+        </is>
+      </c>
+    </row>
+    <row r="38"/>
+    <row r="39"/>
+    <row r="40"/>
+    <row r="41"/>
+    <row r="42"/>
+    <row r="43"/>
+    <row r="44"/>
+    <row r="45"/>
+    <row r="46"/>
+    <row r="47"/>
+    <row r="48"/>
+    <row r="49"/>
+    <row r="50"/>
+    <row r="51"/>
+    <row r="52"/>
+    <row r="53"/>
+    <row r="54"/>
+    <row r="55"/>
+    <row r="56"/>
+    <row r="57"/>
+    <row r="58"/>
+    <row r="59"/>
+    <row r="60"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1728,7 +2297,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B9"/>
+  <dimension ref="A1:B20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1743,89 +2312,100 @@
       </c>
     </row>
     <row r="3" ht="30" customHeight="1">
-      <c r="A3" s="12" t="inlineStr">
+      <c r="A3" s="15" t="inlineStr">
         <is>
           <t>動作環境</t>
         </is>
       </c>
       <c r="B3" s="13" t="inlineStr">
         <is>
-          <t>Docker / Docker Compose(推奨)、または Node.js 18以上 + Ollama をローカルにインストールした環境。</t>
+          <t>Docker / Docker Compose(推奨)、または Node.js 18以上 + Ollama をローカルにインストールした環境。社内向け本番運用の場合はIDCFクラウド等の仮想マシンまたはKubernetesクラスタ上での稼働を想定(DEPLOY_IDCF.md/DEPLOY_K8S.md参照)。</t>
         </is>
       </c>
     </row>
     <row r="4" ht="30" customHeight="1">
-      <c r="A4" s="12" t="inlineStr">
+      <c r="A4" s="15" t="inlineStr">
         <is>
           <t>対応ブラウザ</t>
         </is>
       </c>
       <c r="B4" s="13" t="inlineStr">
         <is>
-          <t>主要モダンブラウザ(Chrome, Edge, Safari, Firefox 等の最新版)を想定。fetch のストリーミングAPI(ReadableStream)に対応していることが前提。</t>
+          <t>主要モダンブラウザ(Chrome, Edge, Safari, Firefox等の最新版)を想定。ドラッグ&amp;ドロップAPI・fetchによるmultipart送信に対応していることが前提。</t>
         </is>
       </c>
     </row>
     <row r="5" ht="20" customHeight="1">
-      <c r="A5" s="12" t="inlineStr">
+      <c r="A5" s="15" t="inlineStr">
         <is>
           <t>可用性・利用形態</t>
         </is>
       </c>
       <c r="B5" s="13" t="inlineStr">
         <is>
-          <t>単一ユーザー・単一プロセスでのローカル利用を想定。外部公開や同時多接続は想定していない。</t>
+          <t>ローカル環境では単一ユーザーでの利用を想定。社内向け本番構成では、社内ネットワーク/VPN限定のアクセス制限とGoogle Workspace SSOを組み合わせ、複数ユーザーが同一サーバーを共有する運用を想定(同時に重い個人情報チェックが複数実行されるとCPUのみの環境では応答が遅くなる点に留意)。</t>
         </is>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1">
-      <c r="A6" s="12" t="inlineStr">
+      <c r="A6" s="15" t="inlineStr">
         <is>
           <t>セキュリティ</t>
         </is>
       </c>
       <c r="B6" s="13" t="inlineStr">
         <is>
-          <t>認証・認可の仕組みは実装していない。ローカルホストでの利用を前提とし、外部ネットワークへの公開は推奨しない。</t>
+          <t>アプリ自体には認証・認可の仕組みを実装していない。ローカル利用時はローカルホストでの利用を前提とし外部公開は推奨しない。社内向け本番構成ではoauth2-proxyによるGoogle Workspace認証とネットワークレベルのアクセス制限(社内/VPN限定)の2段構えで保護する。アップロードされたファイルの内容や検出された個人情報の中身はサーバーに保存されない(アップロード監査ログにも含まれない)。</t>
         </is>
       </c>
     </row>
     <row r="7" ht="30" customHeight="1">
-      <c r="A7" s="12" t="inlineStr">
+      <c r="A7" s="15" t="inlineStr">
         <is>
           <t>パフォーマンス</t>
         </is>
       </c>
       <c r="B7" s="13" t="inlineStr">
         <is>
-          <t>応答速度はOllamaでのモデル推論性能(ホストのCPU/GPU、使用モデルサイズ)に依存する。GPU利用時は docker-compose.yml のNVIDIA GPU設定を有効化することで高速化できる。</t>
+          <t>応答速度はOllamaでのモデル推論性能(ホストのCPU/GPU、使用モデルサイズ)に依存する。既定モデルgemma4:e4bはCPUのみの環境でも比較的高速に動作するよう選定している。より大きいモデル(gemma4:12b等)を使う場合は応答が数分かかることがあるため、OLLAMA_TIMEOUT_MS・PII_CHUNK_CHAR_LIMIT等での調整や、本番構成ではoauth2-proxyのOAUTH2_PROXY_UPSTREAM_TIMEOUT延長(既定30秒のままでは502 Bad Gatewayになる)が必要。GPU利用時はdocker-compose.ymlのNVIDIA GPU設定を有効化することで高速化できる。</t>
         </is>
       </c>
     </row>
     <row r="8" ht="45" customHeight="1">
-      <c r="A8" s="12" t="inlineStr">
+      <c r="A8" s="15" t="inlineStr">
         <is>
           <t>データ永続性</t>
         </is>
       </c>
       <c r="B8" s="13" t="inlineStr">
         <is>
-          <t>会話履歴はブラウザのlocalStorageにのみ保存され、サーバー再起動の影響は受けないが、ブラウザ側のデータ消去で失われる。モデルデータはDockerボリューム(ollama_data)により、コンテナ再作成後も保持される。</t>
+          <t>アップロードされたファイルの内容・検出結果はメモリ上でのみ処理され保存されない。モデルデータはDockerボリューム(ollama_data)、アップロード監査ログはDockerボリューム(pii_logs)により、コンテナ再作成後も保持される(既定90日経過分は自動削除)。</t>
         </is>
       </c>
     </row>
     <row r="9" ht="20" customHeight="1">
-      <c r="A9" s="12" t="inlineStr">
+      <c r="A9" s="15" t="inlineStr">
         <is>
           <t>保守性</t>
         </is>
       </c>
       <c r="B9" s="13" t="inlineStr">
         <is>
-          <t>サーバー・フロントエンドともに外部フレームワークへの依存を最小限に抑え、小規模な構成を維持している。</t>
-        </is>
-      </c>
-    </row>
+          <t>サーバー・フロントエンドともに外部フレームワークへの依存を最小限に抑え、ファイル形式ごとの解析処理はlib/pii.jsに、監査ログ処理はlib/auditLog.jsに分離している。</t>
+        </is>
+      </c>
+    </row>
+    <row r="10"/>
+    <row r="11"/>
+    <row r="12"/>
+    <row r="13"/>
+    <row r="14"/>
+    <row r="15"/>
+    <row r="16"/>
+    <row r="17"/>
+    <row r="18"/>
+    <row r="19"/>
+    <row r="20"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1837,7 +2417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C8"/>
+  <dimension ref="A1:C20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1853,97 +2433,123 @@
       </c>
     </row>
     <row r="3" ht="22" customHeight="1">
-      <c r="A3" s="8" t="inlineStr">
+      <c r="A3" s="16" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="B3" s="8" t="inlineStr">
+      <c r="B3" s="16" t="inlineStr">
         <is>
           <t>項目</t>
         </is>
       </c>
-      <c r="C3" s="8" t="inlineStr">
+      <c r="C3" s="16" t="inlineStr">
         <is>
           <t>内容</t>
         </is>
       </c>
     </row>
     <row r="4" ht="50" customHeight="1">
-      <c r="A4" s="9" t="n">
+      <c r="A4" s="17" t="n">
         <v>1</v>
       </c>
-      <c r="B4" s="9" t="inlineStr">
-        <is>
-          <t>gemma4タグの実在確認</t>
+      <c r="B4" s="17" t="inlineStr">
+        <is>
+          <t>画像内文字の非対応</t>
         </is>
       </c>
       <c r="C4" s="10" t="inlineStr">
         <is>
-          <t>本仕様書作成時点でOllamaのモデルライブラリに "gemma4" タグが実在するか未確認。存在しない場合は "gemma3" 等の実在するタグを MODEL_NAME に設定して利用する運用となる。</t>
+          <t>スキャン画像のみのPDF、docx/pptx内の画像に含まれる文字は現時点でテキスト抽出・検出の対象外(OCR機能は未実装)。目視での確認が必要。</t>
         </is>
       </c>
     </row>
     <row r="5" ht="50" customHeight="1">
-      <c r="A5" s="9" t="n">
+      <c r="A5" s="17" t="n">
         <v>2</v>
       </c>
-      <c r="B5" s="9" t="inlineStr">
-        <is>
-          <t>サーバーサイドでの会話履歴永続化</t>
+      <c r="B5" s="17" t="inlineStr">
+        <is>
+          <t>docx/pptxの表構造検出</t>
         </is>
       </c>
       <c r="C5" s="10" t="inlineStr">
         <is>
-          <t>現状はブラウザのlocalStorageのみに保存されるため、別端末・別ブラウザ間での履歴共有ができない。必要であればDB等を用いたサーバー側保存への拡張を検討する。</t>
+          <t>docx/pptxの表の文字自体は抽出されるが、xlsx/csv/pdf罫線表のような列見出しによる機械的なカテゴリ判定(機能一覧No.3)は構造情報を保持していないため対象外。パターン検出・ラベル検出・AI検出のみで判定する。</t>
         </is>
       </c>
     </row>
     <row r="6" ht="50" customHeight="1">
-      <c r="A6" s="9" t="n">
+      <c r="A6" s="17" t="n">
         <v>3</v>
       </c>
-      <c r="B6" s="9" t="inlineStr">
-        <is>
-          <t>認証・アクセス制御</t>
+      <c r="B6" s="17" t="inlineStr">
+        <is>
+          <t>人物名パターン検出の網羅性</t>
         </is>
       </c>
       <c r="C6" s="10" t="inlineStr">
         <is>
-          <t>現状は認証機構を持たないため、ローカル利用を前提としている。社内サーバー等複数人がアクセスする環境で利用する場合は、認証機能の追加を検討する。</t>
+          <t>敬称なしの人物名検出は、あらかじめ登録した約140種の代表的な日本人の名字のみを手がかりにしており、リストにない名字(珍しい名字・外国人名等)は検出できない。網羅的な検出にはAI判定の精度向上が必要。</t>
         </is>
       </c>
     </row>
     <row r="7" ht="50" customHeight="1">
-      <c r="A7" s="9" t="n">
+      <c r="A7" s="17" t="n">
         <v>4</v>
       </c>
-      <c r="B7" s="9" t="inlineStr">
-        <is>
-          <t>モデル取得の自動化</t>
+      <c r="B7" s="17" t="inlineStr">
+        <is>
+          <t>Kubernetes構成のoauth2-proxyタイムアウト設定</t>
         </is>
       </c>
       <c r="C7" s="10" t="inlineStr">
         <is>
-          <t>現状は初回に手動で `docker compose exec ollama ollama pull &lt;model&gt;` を実行する必要がある。起動時に自動でモデルを取得する仕組みがあると利便性が向上する。</t>
+          <t>docker-compose.prod.ymlには個人情報チェックの長時間応答に対応するOAUTH2_PROXY_UPSTREAM_TIMEOUT設定を追加済みだが、k8s/08-oauth2-proxy-deployment.yamlには未反映(別タスクとして切り出し済み)。k8s環境では502 Bad Gatewayが再発する可能性がある。</t>
         </is>
       </c>
     </row>
     <row r="8" ht="50" customHeight="1">
-      <c r="A8" s="9" t="n">
+      <c r="A8" s="17" t="n">
         <v>5</v>
       </c>
-      <c r="B8" s="9" t="inlineStr">
-        <is>
-          <t>実機での動作確認</t>
+      <c r="B8" s="17" t="inlineStr">
+        <is>
+          <t>ログインユーザー名の信頼性</t>
         </is>
       </c>
       <c r="C8" s="10" t="inlineStr">
         <is>
-          <t>本仕様書の内容は開発環境上のコード確認・簡易テストに基づく。実際のOllama/Gemmaモデルおよび docker compose up による本番相当環境での動作確認が必要。</t>
-        </is>
-      </c>
-    </row>
+          <t>アップロード監査ログのユーザー名は、appに直接到達できる構成(認証なしのローカル開発環境等)ではクライアントが送信するヘッダー値をそのまま信用する実装のため、偽装が可能。oauth2-proxy経由でのみappに到達できる構成(本番・認証確認用)でのみ信頼できる値となる。</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="17" t="n">
+        <v>6</v>
+      </c>
+      <c r="B9" s="17" t="inlineStr">
+        <is>
+          <t>実運用環境での動作確認</t>
+        </is>
+      </c>
+      <c r="C9" s="10" t="inlineStr">
+        <is>
+          <t>本仕様書の内容は開発環境上のコード確認・ローカルでの動作確認に基づく。IDCFクラウド(VM/Kubernetes)等の実運用環境での負荷・複数ユーザー同時アクセス時の動作確認が必要。</t>
+        </is>
+      </c>
+    </row>
+    <row r="10"/>
+    <row r="11"/>
+    <row r="12"/>
+    <row r="13"/>
+    <row r="14"/>
+    <row r="15"/>
+    <row r="16"/>
+    <row r="17"/>
+    <row r="18"/>
+    <row r="19"/>
+    <row r="20"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>